<commit_message>
Weekly COCHE update 2026-08-24
</commit_message>
<xml_diff>
--- a/COCHE_Papers.xlsx
+++ b/COCHE_Papers.xlsx
@@ -865,55 +865,55 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>42481379</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Ag-Anchored Ti</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>10.1021/acsabm.5c02536</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>ACS applied bio materials</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Bangul Khan, Bilawal Khan, Weibin Zhu, Changqiu Zhou, Ching Yin Fong, Rafi U Shan Ahmad, Iyappan Gunasekran, Mohamed Elhousseini Hilal*, Bee Luan Khoo*</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Bangul Khan, Weibin Zhu, Rafi U Shan Ahmad, Iyappan Gunasekran, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>COCHE affiliation</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>COCHE affiliation</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>ITC 2026</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsabm.5c02536</t>
         </is>

</xml_diff>

<commit_message>
Weekly COCHE update 2026-10-05
</commit_message>
<xml_diff>
--- a/COCHE_Papers.xlsx
+++ b/COCHE_Papers.xlsx
@@ -759,55 +759,55 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>42696383</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Sample-to-Answer Quantitative Rapid Test for Point-of-Care Monitoring of Urinary Cystatin C Levels.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>10.1021/acssensors.6c02077</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>ACS sensors</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Lok Tim Pang, Miu Ling Lam, Cheuk Chun Szeto, Ting-Hsuan Chen*</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Ting-Hsuan Chen</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>COCHE affiliation</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>COCHE affiliation</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>ITC 2026</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acssensors.6c02077</t>
         </is>

</xml_diff>